<commit_message>
Remove Detailed Breakdown sheet from 20h estimate xlsx
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Estimate-TT-AIM-SPRINT-8C-20h.xlsx
+++ b/docs/Estimate-TT-AIM-SPRINT-8C-20h.xlsx
@@ -10,7 +10,6 @@
     <sheet name="Commercial (Met meerwerk)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Estimate" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="CostOf Work" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Detailed Breakdown" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1076,564 +1075,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="100" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>DETAILED BREAKDOWN — TT-AIM-SPRINT-8C (20h Technical Analysis)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Phase</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>Estimate (hours)</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>Environment Setup</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Access and review source code (PHP backend, React frontend, Python LPB app)</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Set up local dev environment (PHP/Slim API, React JS, Python services)</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Restore database snapshot and connect services</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Verify system starts and key workflows function</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Subtotal Phase 1</t>
-        </is>
-      </c>
-      <c r="E7" s="7">
-        <f>SUM(E3:E6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Code &amp; Architecture Review</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Review PHP/Slim API codebase structure and patterns</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Review React JS frontend architecture</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Review Python LPB application and data pipeline</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Database schema analysis (terminals, ships, subscriptions, benchmarking data)</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Map external integrations (Stripe subscriptions, ReCaptcha, APIs, email)</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Infrastructure &amp; deployment review (staging/production, DevOps setup)</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Subtotal Phase 2</t>
-        </is>
-      </c>
-      <c r="E15" s="7">
-        <f>SUM(E9:E14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>TT-2436</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Security &amp; anti-abuse</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>Review login tracking, CSRF, ReCaptcha integration points</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Original est: 12h</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>TT-2439</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>LPB / Python pipeline</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Assess berth data function, asset class extensibility</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Original est: 20h</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>TT-2434</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Subscription splitting</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>Map Stripe vs non-Stripe logic, data migration needs</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Original est: 3.5h</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>TT-2423</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Logical Checks Dashboard</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>Evaluate 30 rules engine, dashboard architecture, tab layout complexity</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Original est: 58.5h</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>TT-2444</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Rhine CPP API</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>Review back-office gasoil/gasoline data flow and API exposure</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>Original est: 4h</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>TT-2435</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Ship &amp; Terminal Modal</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Assess factsheet UI, map integration, berth widget, responsive constraints</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Original est: 64h</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>TT-2443</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Historical Waiting Times</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Evaluate data processing pipeline requirements</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Original est: TBD</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Cross-ticket dependency analysis and strategy recommendation</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Subtotal Phase 3</t>
-        </is>
-      </c>
-      <c r="E25" s="7">
-        <f>SUM(E17:E24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Risk Assessment</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Stripe integration complexity &amp; subscription data migration risks</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>Rules engine scalability &amp; dashboard performance (TT-2423)</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>Python LPB pipeline changes impacting existing data (TT-2439)</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>Security implementation gaps (CSRF, ReCaptcha, abuse detection)</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Mobile/responsive UI constraints (TT-2435)</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Define mitigation strategies and testing approach</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="n">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>Subtotal Phase 4</t>
-        </is>
-      </c>
-      <c r="E33" s="7">
-        <f>SUM(E27:E32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>Reporting</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>Compile findings into technical analysis report</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="n">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>Prepare prioritized implementation roadmap with dependencies</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>Review and finalize deliverables</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>Subtotal Reporting</t>
-        </is>
-      </c>
-      <c r="E38" s="7">
-        <f>SUM(E35:E37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL ANALYSIS HOURS</t>
-        </is>
-      </c>
-      <c r="E40" s="7">
-        <f>SUM(E3:E37)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="B9:B14"/>
-    <mergeCell ref="A9:A14"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="A17:A24"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="B3:B6"/>
-    <mergeCell ref="B27:B32"/>
-    <mergeCell ref="A27:A32"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>